<commit_message>
Corrected ZIF orientation and started 3D designs
</commit_message>
<xml_diff>
--- a/UHDEMG/07 - EXPORTS/BOM/UHDEMG_BOM.xlsx
+++ b/UHDEMG/07 - EXPORTS/BOM/UHDEMG_BOM.xlsx
@@ -1,26 +1,125 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olivi\Documents\Universite Laval\Maitrise\Projet\UHDEMG\UHDEMG\07 - EXPORTS\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5676AF0B-82EB-42D6-9C61-E48F846F1A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-28755" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="4" r:id="rId1"/>
+    <sheet name="PCBWAY" sheetId="1" r:id="rId2"/>
+    <sheet name="Digikey &amp; INTAN" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="25">
+  <si>
+    <t>Project Name</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Cost (CAD)</t>
+  </si>
+  <si>
+    <t>PCBWAY Quote Parameters</t>
+  </si>
+  <si>
+    <t>DB_Panel</t>
+  </si>
+  <si>
+    <t>Microneedle_Patch</t>
+  </si>
+  <si>
+    <t>Microneedle_Patch_Mirrored</t>
+  </si>
+  <si>
+    <t>RHD2132_64CH</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Parameter</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Cart Link</t>
+  </si>
+  <si>
+    <t>Cart Cost</t>
+  </si>
+  <si>
+    <t>Cart Currency</t>
+  </si>
+  <si>
+    <t>Digikey</t>
+  </si>
+  <si>
+    <t>INTAN</t>
+  </si>
+  <si>
+    <t>Part Number</t>
+  </si>
+  <si>
+    <t>Unit Cost</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
+  </si>
+  <si>
+    <t>Total Cost (CAD)</t>
+  </si>
+  <si>
+    <t>Cost Summary</t>
+  </si>
+  <si>
+    <t>PCBWAY</t>
+  </si>
+  <si>
+    <t>Supplier</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,13 +127,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +162,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +448,241 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0A50ECAC-6578-4F5C-AA70-A9524ED3CD1E}">
+  <dimension ref="C3:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C7" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11">
+        <f>SUM(D7:D9)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:T9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="26.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="2.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" customWidth="1"/>
+    <col min="11" max="11" width="13.33203125" customWidth="1"/>
+    <col min="13" max="13" width="12.33203125" customWidth="1"/>
+    <col min="14" max="14" width="12.6640625" customWidth="1"/>
+    <col min="16" max="16" width="12.5546875" customWidth="1"/>
+    <col min="17" max="17" width="16.6640625" customWidth="1"/>
+    <col min="19" max="20" width="12.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="I2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="M4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="N4" s="2"/>
+      <c r="P4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="2"/>
+      <c r="S4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="T4" s="2"/>
+    </row>
+    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" t="s">
+        <v>10</v>
+      </c>
+      <c r="K5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M5" t="s">
+        <v>10</v>
+      </c>
+      <c r="N5" t="s">
+        <v>11</v>
+      </c>
+      <c r="P5" t="s">
+        <v>10</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>11</v>
+      </c>
+      <c r="S5" t="s">
+        <v>10</v>
+      </c>
+      <c r="T5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9">
+        <f>SUM(E4:E7)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48B8B8C0-6332-43EC-B796-9B1BE59D0815}">
+  <dimension ref="B4:B21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" ht="21" x14ac:dyDescent="0.4">
+      <c r="B14" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>